<commit_message>
clean up on instructional pages
</commit_message>
<xml_diff>
--- a/static/pages/course_model/ml05-ols/regression-simple-error-spreadsheet.xlsx
+++ b/static/pages/course_model/ml05-ols/regression-simple-error-spreadsheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ndg00008/Library/CloudStorage/Dropbox/Obsidian/courses/course_model/ml05-ols/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ndg00008/Documents/profgarrett/jsgames/static/pages/course_model/ml05-ols/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B78A066-969F-424B-8648-D1D7C1E43AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F144DC05-97FF-4F41-AFCC-9EA071FAB18A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-77960" yWindow="-1800" windowWidth="27040" windowHeight="15820" xr2:uid="{4E0B4222-6DFF-E149-A11D-AB042D352AA1}"/>
+    <workbookView xWindow="1600" yWindow="660" windowWidth="27040" windowHeight="15820" xr2:uid="{4E0B4222-6DFF-E149-A11D-AB042D352AA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,16 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
-  <si>
-    <t>a</t>
-  </si>
-  <si>
-    <t>b</t>
-  </si>
-  <si>
-    <t>c</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t>x</t>
   </si>
@@ -65,20 +56,47 @@
     <t>dif</t>
   </si>
   <si>
-    <t>rmse</t>
-  </si>
-  <si>
-    <t>d</t>
-  </si>
-  <si>
     <t>avg</t>
+  </si>
+  <si>
+    <t>Alice</t>
+  </si>
+  <si>
+    <t>Bob</t>
+  </si>
+  <si>
+    <t>Charlie</t>
+  </si>
+  <si>
+    <t>David</t>
+  </si>
+  <si>
+    <t>years worked</t>
+  </si>
+  <si>
+    <t>salary</t>
+  </si>
+  <si>
+    <t>y = 5x + 30</t>
+  </si>
+  <si>
+    <t>sse</t>
+  </si>
+  <si>
+    <t>rsme</t>
+  </si>
+  <si>
+    <t>sst</t>
+  </si>
+  <si>
+    <t>r^2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -90,6 +108,13 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -188,7 +213,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -208,6 +233,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -542,190 +568,220 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FB54C0E-2D07-AB4B-9132-089D2399FCA2}">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="8" width="8.33203125" customWidth="1"/>
+    <col min="1" max="1" width="8.33203125" customWidth="1"/>
+    <col min="2" max="2" width="12.1640625" customWidth="1"/>
+    <col min="3" max="8" width="8.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
         <v>3</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F3" t="s">
         <v>4</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G3" t="s">
         <v>5</v>
       </c>
-      <c r="E1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1">
-        <v>0</v>
-      </c>
-      <c r="C2" s="2">
-        <v>30</v>
-      </c>
-      <c r="D2" s="2">
-        <v>30</v>
-      </c>
-      <c r="E2">
-        <f>C2-D2</f>
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <f>E2*E2</f>
-        <v>0</v>
-      </c>
-      <c r="G2">
-        <f>C2-$C$7</f>
-        <v>-13.333333333333336</v>
-      </c>
-      <c r="H2">
-        <f>G2*G2</f>
-        <v>177.77777777777783</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="3">
-        <v>2</v>
-      </c>
-      <c r="C3" s="4">
-        <v>40</v>
-      </c>
-      <c r="D3" s="4">
-        <v>40</v>
-      </c>
-      <c r="E3">
-        <f>C3-D3</f>
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <f>E3*E3</f>
-        <v>0</v>
-      </c>
-      <c r="G3">
-        <f>C3-$C$7</f>
-        <v>-3.3333333333333357</v>
-      </c>
-      <c r="H3">
-        <f>G3*G3</f>
-        <v>11.111111111111127</v>
+      <c r="H3" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="3">
-        <v>4</v>
-      </c>
-      <c r="C4" s="4">
-        <v>60</v>
-      </c>
-      <c r="D4" s="4">
-        <v>50</v>
+        <v>7</v>
+      </c>
+      <c r="B4" s="1">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2">
+        <v>30</v>
+      </c>
+      <c r="D4" s="2">
+        <f>30+5*B4</f>
+        <v>30</v>
       </c>
       <c r="E4">
-        <f>C4-D4</f>
-        <v>10</v>
+        <f>D4-C4</f>
+        <v>0</v>
       </c>
       <c r="F4">
         <f>E4*E4</f>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <f>C4-$C$7</f>
-        <v>16.666666666666664</v>
+        <f>C4-$C$9</f>
+        <v>-12.5</v>
       </c>
       <c r="H4">
         <f>G4*G4</f>
-        <v>277.77777777777771</v>
+        <v>156.25</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="5">
-        <v>4</v>
-      </c>
-      <c r="C5" s="6">
+        <v>8</v>
+      </c>
+      <c r="B5" s="3">
+        <v>2</v>
+      </c>
+      <c r="C5" s="4">
         <v>40</v>
       </c>
-      <c r="D5" s="6">
-        <v>50</v>
+      <c r="D5" s="2">
+        <f>30+5*B5</f>
+        <v>40</v>
       </c>
       <c r="E5">
-        <f>C5-D5</f>
-        <v>-10</v>
+        <f>D5-C5</f>
+        <v>0</v>
       </c>
       <c r="F5">
         <f>E5*E5</f>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <f>C5-$C$7</f>
-        <v>-3.3333333333333357</v>
+        <f>C5-$C$9</f>
+        <v>-2.5</v>
       </c>
       <c r="H5">
         <f>G5*G5</f>
-        <v>11.111111111111127</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7">
-        <f>AVERAGE(C2:C4)</f>
-        <v>43.333333333333336</v>
-      </c>
-      <c r="E7" t="s">
+        <v>6.25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>9</v>
       </c>
+      <c r="B6" s="3">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4">
+        <v>60</v>
+      </c>
+      <c r="D6" s="2">
+        <f>30+5*B6</f>
+        <v>50</v>
+      </c>
+      <c r="E6">
+        <f>D6-C6</f>
+        <v>-10</v>
+      </c>
+      <c r="F6">
+        <f>E6*E6</f>
+        <v>100</v>
+      </c>
+      <c r="G6">
+        <f>C6-$C$9</f>
+        <v>17.5</v>
+      </c>
+      <c r="H6">
+        <f>G6*G6</f>
+        <v>306.25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="5">
+        <v>4</v>
+      </c>
+      <c r="C7" s="6">
+        <v>40</v>
+      </c>
+      <c r="D7" s="2">
+        <f>30+5*B7</f>
+        <v>50</v>
+      </c>
+      <c r="E7">
+        <f>D7-C7</f>
+        <v>10</v>
+      </c>
       <c r="F7">
-        <f>SUM(F2:F5)</f>
+        <f>E7*E7</f>
+        <v>100</v>
+      </c>
+      <c r="G7">
+        <f>C7-$C$9</f>
+        <v>-2.5</v>
+      </c>
+      <c r="H7">
+        <f>G7*G7</f>
+        <v>6.25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="E8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="7">
+        <f>SUM(F4:F7)</f>
         <v>200</v>
       </c>
-      <c r="H7">
-        <f>SUM(H2:H5)</f>
-        <v>477.77777777777777</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="F8">
-        <f>AVERAGE(F2:F5)</f>
+      <c r="G8" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" s="7">
+        <f>SUM(H4:H7)</f>
+        <v>475</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9">
+        <f>AVERAGE(C4:C7)</f>
+        <v>42.5</v>
+      </c>
+      <c r="E9" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9">
+        <f>AVERAGE(F4:F7)</f>
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="F9">
-        <f>SQRT(F8)</f>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10">
+        <f>SQRT(F9)</f>
         <v>7.0710678118654755</v>
       </c>
-      <c r="H9">
-        <f>1-(200/478)</f>
-        <v>0.58158995815899583</v>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12">
+        <f>1 - (F8/H8)</f>
+        <v>0.57894736842105265</v>
       </c>
     </row>
   </sheetData>

</xml_diff>